<commit_message>
v2.7.2 : vrais modeles Excel + regles R1-R10 + corrections retours reels
- Bascule sur les vrais modeles (bungalows, sanitaires, container, cuve)
- Regles metier R1-R10 (assemblage, doses, elingage, climatisation, fonction)
- Nouveau module app/regles_modeles.py (+ tests/test_regles_modeles.py)
- CUVE branchee ; lave-mains retire ; correspondances/cellules a jour
- Docs de suivi (PLAN_CORRECTIONS, RETOURS_TESTS_BOSS, MODELES_CELLULES_REFERENCE)
- Lanceur 'derniere version' depuis les sources (contournement antivirus)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/polysani_handi.xlsx
+++ b/templates/polysani_handi.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Joris\gb-etats-des-lieux\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Joris\gb-etats-des-lieux\modeles_reels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CEBD5C5-54D8-4100-8D9E-FB0161C98C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3A00EE2-3E43-4134-A61C-E4B44F17A573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2595" yWindow="2595" windowWidth="21600" windowHeight="12660" xr2:uid="{927CC8A1-6FB2-476B-AE4C-A5D6B527708D}"/>
+    <workbookView xWindow="2595" yWindow="2595" windowWidth="21600" windowHeight="12660" activeTab="3" xr2:uid="{927CC8A1-6FB2-476B-AE4C-A5D6B527708D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Polysani H" sheetId="1" r:id="rId1"/>
+    <sheet name="3 WCH" sheetId="4" r:id="rId1"/>
+    <sheet name="Polysani H" sheetId="1" r:id="rId2"/>
+    <sheet name="Polysani H S13542" sheetId="5" r:id="rId3"/>
+    <sheet name="Poly H containex S22325 OU 326 " sheetId="9" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="67">
   <si>
     <t>ETAT INTERIEUR</t>
   </si>
@@ -162,6 +165,12 @@
     <t>CHENEAUX NETTOYES   OUI    NON</t>
   </si>
   <si>
+    <t>CLIENT :</t>
+  </si>
+  <si>
+    <t>W ….…………..…..</t>
+  </si>
+  <si>
     <t>OUI</t>
   </si>
   <si>
@@ -174,20 +183,68 @@
     <t>Nom préparateur :                                         Visa contrôleur :                                          Date :</t>
   </si>
   <si>
+    <t>Sanitaire : 3WC HANDI</t>
+  </si>
+  <si>
     <t>S ….…………..…..</t>
   </si>
   <si>
     <t>Sanitaire : 5WC / 3UR (POLYSANI HANDI)</t>
   </si>
   <si>
+    <t>S 13542</t>
+  </si>
+  <si>
+    <t>CLEF CLOISONS INTERIEURES :  OUI     NON</t>
+  </si>
+  <si>
+    <t>CLEF BLOC SANI :  OUI        NON</t>
+  </si>
+  <si>
+    <t>Dévidoir papier
+Type Jumbo + Clé</t>
+  </si>
+  <si>
+    <t>Produit nettoyage pour urinoirs</t>
+  </si>
+  <si>
+    <t>3 Urinoirs (sans eau)</t>
+  </si>
+  <si>
     <t xml:space="preserve">CLIENT : </t>
+  </si>
+  <si>
+    <t>Lavabo + robinets + chauffe eau</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> + groom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nom préparateur :    
+Visa contrôleur :                                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° CE :   
+CLEF :  OUI      NON                                              </t>
+  </si>
+  <si>
+    <t>S 22326</t>
+  </si>
+  <si>
+    <t>S 22325</t>
+  </si>
+  <si>
+    <t>CHANTIER :</t>
+  </si>
+  <si>
+    <t>Sanitaire : 5WC / 2UR (POLYSANI HANDI)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -246,8 +303,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -260,8 +329,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -545,6 +620,19 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -553,9 +641,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -565,11 +654,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -624,7 +720,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -666,68 +762,140 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -735,7 +903,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
@@ -747,41 +915,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,6 +978,350 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>809625</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4260" name="Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6CBC4F6-822B-7422-3FAA-6104AEDF099C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4229100" y="2228850"/>
+          <a:ext cx="1600200" cy="1295400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4261" name="Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9736A119-FA9C-C2A1-47AD-03A43BBDBFA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="723900" y="2276475"/>
+          <a:ext cx="1600200" cy="1247775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Text Box 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64A98129-3FB7-6486-6F37-076890259E6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3248025" y="161925"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>PIGNON </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Text Box 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FA104E9-BDBC-9DE5-0BDE-49EED8F35788}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="304800" y="161925"/>
+          <a:ext cx="657225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>Longpan AV</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4264" name="Image 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{470A7A14-4486-FF12-5622-22BB4DF899F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect b="24324"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="19050" y="47625"/>
+          <a:ext cx="2733675" cy="600075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -1285,6 +1806,768 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11313" name="Image 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDDD98FE-3E67-35FC-5C83-47DE572082A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect b="24324"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="57150" y="66675"/>
+          <a:ext cx="2733675" cy="600075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11314" name="Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF2F9362-278F-DB68-01A4-EEC50D1D8893}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3486150" y="2571750"/>
+          <a:ext cx="2371725" cy="1085850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11315" name="Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5649354B-12AB-A31C-0BF5-A36DFD500495}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="38100" y="2571750"/>
+          <a:ext cx="2362200" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Text Box 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E503D423-9D38-2FF6-BAD1-E3A09DE956F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3190875" y="0"/>
+          <a:ext cx="0" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>PIGNON </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Text Box 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18336583-3EFF-79A5-A597-2E9A1E9B2148}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6848475" y="0"/>
+          <a:ext cx="0" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>Longpan AR</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>866775</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13363" name="Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D24604E5-E2C3-5F80-7D34-72F060E32A8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3514725" y="4438650"/>
+          <a:ext cx="2371725" cy="1085850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13364" name="Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96E5DBCB-17D0-F59C-2110-A8B92483BCF6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="66675" y="4438650"/>
+          <a:ext cx="2362200" cy="1047750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+        <a:scene3d>
+          <a:camera prst="legacyPerspectiveFront">
+            <a:rot lat="600000" lon="2100000" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="legacyFlat2" dir="b"/>
+        </a:scene3d>
+        <a:sp3d extrusionH="1801800" prstMaterial="legacyMatte">
+          <a:bevelT w="13500" h="13500" prst="angle"/>
+          <a:bevelB w="13500" h="13500" prst="angle"/>
+          <a:extrusionClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:extrusionClr>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Text Box 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADB39AF8-4DD9-BAB4-0079-F173DB8F362A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3190875" y="161925"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>PIGNON </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>D</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Text Box 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00C7C6B5-1536-FAF3-E3FD-B321ECBDC0D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="304800" y="161925"/>
+          <a:ext cx="657225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:rPr>
+            <a:t>Longpan AV</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13367" name="Image 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E9584CB-DA77-6674-552B-E013F600E41F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect b="24324"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="66675" y="114300"/>
+          <a:ext cx="2733675" cy="600075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>847725</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>1209675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13368" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EF440C4-E7CE-D620-FBC8-8F92EEBD3A15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="17786" t="28021" r="35115" b="25682"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2743200" y="1409700"/>
+          <a:ext cx="4038600" cy="2228850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -1632,652 +2915,1419 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE975CBE-29B4-43BA-961C-66ECCC4AF27C}">
+  <sheetPr codeName="Feuil3">
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:H59"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" style="8"/>
+    <col min="2" max="2" width="9" style="8" customWidth="1"/>
+    <col min="3" max="8" width="13.7109375" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E2" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+    </row>
+    <row r="3" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+    </row>
+    <row r="4" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E5" s="84" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="86" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="86"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="97"/>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97"/>
+    </row>
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="16"/>
+      <c r="E7" s="84" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
+    </row>
+    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="D8" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="85" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="85"/>
+    </row>
+    <row r="9" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="78" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="78"/>
+      <c r="C9" s="78"/>
+      <c r="D9" s="78"/>
+      <c r="E9" s="78"/>
+      <c r="F9" s="78"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="78"/>
+    </row>
+    <row r="10" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
+      <c r="H10" s="68"/>
+    </row>
+    <row r="11" spans="1:8" ht="2.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="96" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="93"/>
+      <c r="B19" s="93"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="94" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="95"/>
+      <c r="C24" s="79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="80"/>
+      <c r="E24" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="29"/>
+      <c r="G24" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="21"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="75"/>
+      <c r="E25" s="68"/>
+      <c r="F25" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="75"/>
+      <c r="H25" s="68"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H26" s="28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="87"/>
+      <c r="C27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="88"/>
+      <c r="B28" s="89"/>
+      <c r="C28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="90"/>
+      <c r="C29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="91"/>
+      <c r="B30" s="92"/>
+      <c r="C30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="79" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="80"/>
+      <c r="C31" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="82"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="82"/>
+      <c r="H31" s="83"/>
+    </row>
+    <row r="32" spans="1:8" s="1" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="42"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="70"/>
+      <c r="C33" s="70"/>
+      <c r="D33" s="70"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="70"/>
+      <c r="G33" s="70"/>
+      <c r="H33" s="48"/>
+    </row>
+    <row r="34" spans="1:8" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="75"/>
+      <c r="E34" s="68"/>
+      <c r="F34" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G34" s="75"/>
+      <c r="H34" s="68"/>
+    </row>
+    <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G35" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="72"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+    </row>
+    <row r="37" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="73"/>
+      <c r="B37" s="62"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="61" t="s">
+        <v>28</v>
+      </c>
+      <c r="B38" s="76"/>
+      <c r="C38" s="43"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="76"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" s="76"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+    </row>
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="B41" s="76"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+    </row>
+    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="61" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="76"/>
+      <c r="C42" s="35"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+    </row>
+    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="61" t="s">
+        <v>32</v>
+      </c>
+      <c r="B43" s="76"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B44" s="76"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="61" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" s="76"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" s="76"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="B47" s="76"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="61" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" s="76"/>
+      <c r="C48" s="38"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" s="76"/>
+      <c r="C49" s="38"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="61" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" s="76"/>
+      <c r="C50" s="47"/>
+      <c r="D50" s="39"/>
+      <c r="E50" s="39"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="39"/>
+      <c r="H50" s="39"/>
+    </row>
+    <row r="51" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="B51" s="62"/>
+      <c r="C51" s="37"/>
+      <c r="D51" s="37"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
+    </row>
+    <row r="52" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="B52" s="62"/>
+      <c r="C52" s="34"/>
+      <c r="D52" s="34"/>
+      <c r="E52" s="34"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="35"/>
+    </row>
+    <row r="53" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="63" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" s="64"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="32"/>
+    </row>
+    <row r="54" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B54" s="65"/>
+      <c r="C54" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="20"/>
+    </row>
+    <row r="55" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="66" t="s">
+        <v>37</v>
+      </c>
+      <c r="B55" s="67"/>
+      <c r="C55" s="67"/>
+      <c r="D55" s="67"/>
+      <c r="E55" s="67"/>
+      <c r="F55" s="67"/>
+      <c r="G55" s="67"/>
+      <c r="H55" s="68"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" s="65"/>
+      <c r="C56" s="65"/>
+      <c r="D56" s="65"/>
+      <c r="E56" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="F56" s="65"/>
+      <c r="G56" s="65"/>
+      <c r="H56" s="65"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="60"/>
+      <c r="C58" s="60"/>
+      <c r="D58" s="60"/>
+      <c r="E58" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="F58" s="60"/>
+      <c r="G58" s="60"/>
+      <c r="H58" s="60"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A27:B28"/>
+    <mergeCell ref="A29:B30"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="E2:H4"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A36:B37"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="E58:H58"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="E56:H56"/>
+  </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.18" right="0.15" top="0.17" bottom="0.18" header="0.17" footer="0.18"/>
+  <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C5D1728-3C58-4933-9074-C3D36C5218C8}">
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H58"/>
+  <dimension ref="A2:H59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="5"/>
-    <col min="2" max="2" width="9" style="5" customWidth="1"/>
-    <col min="3" max="8" width="13.7109375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" style="8"/>
+    <col min="2" max="2" width="9" style="8" customWidth="1"/>
+    <col min="3" max="8" width="13.7109375" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E2" s="72" t="s">
+      <c r="E2" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
     </row>
     <row r="3" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
     </row>
     <row r="4" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="72"/>
-      <c r="H4" s="72"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E5" s="73" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
+      <c r="E5" s="84" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
     </row>
     <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="86" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="86"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="97"/>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97"/>
+    </row>
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="16"/>
+      <c r="E7" s="84" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
+    </row>
+    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="D8" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="85" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="85"/>
+    </row>
+    <row r="9" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="78" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="74"/>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="75"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="75"/>
-    </row>
-    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="12"/>
-      <c r="E7" s="73" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="73"/>
-      <c r="G7" s="73"/>
-      <c r="H7" s="73"/>
-    </row>
-    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="D8" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="44"/>
-    </row>
-    <row r="9" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="76" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
+      <c r="B9" s="78"/>
+      <c r="C9" s="78"/>
+      <c r="D9" s="78"/>
+      <c r="E9" s="78"/>
+      <c r="F9" s="78"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="78"/>
     </row>
     <row r="10" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="49"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
+      <c r="H10" s="68"/>
     </row>
     <row r="11" spans="1:8" ht="2.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="69" t="s">
+      <c r="A12" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="69"/>
-      <c r="C12" s="69"/>
-      <c r="D12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
     </row>
     <row r="13" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="41"/>
-      <c r="B19" s="41"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
+      <c r="A19" s="93"/>
+      <c r="B19" s="93"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="3"/>
-      <c r="F22" s="20" t="s">
+      <c r="E22" s="4"/>
+      <c r="F22" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="70" t="s">
+      <c r="A24" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="71"/>
-      <c r="C24" s="57" t="s">
+      <c r="B24" s="95"/>
+      <c r="C24" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="65"/>
-      <c r="E24" s="14" t="s">
+      <c r="D24" s="80"/>
+      <c r="E24" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="14" t="s">
+      <c r="F24" s="29"/>
+      <c r="G24" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="17"/>
+      <c r="H24" s="21"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="52" t="s">
+      <c r="C25" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="D25" s="53"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="52" t="s">
+      <c r="D25" s="75"/>
+      <c r="E25" s="68"/>
+      <c r="F25" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="G25" s="53"/>
-      <c r="H25" s="49"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="68"/>
     </row>
     <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="4" t="s">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="24" t="s">
+      <c r="H26" s="28" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="59"/>
-      <c r="C27" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="F27" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="G27" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="H27" s="21" t="s">
+      <c r="B27" s="87"/>
+      <c r="C27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" s="25" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="60"/>
-      <c r="B28" s="61"/>
-      <c r="C28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="E28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="F28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="G28" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="H28" s="22" t="s">
+      <c r="A28" s="88"/>
+      <c r="B28" s="89"/>
+      <c r="C28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="26" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="62"/>
-      <c r="C29" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D29" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="F29" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H29" s="23" t="s">
+      <c r="B29" s="90"/>
+      <c r="C29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="27" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="63"/>
-      <c r="B30" s="64"/>
-      <c r="C30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E30" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="F30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H30" s="23" t="s">
+      <c r="A30" s="91"/>
+      <c r="B30" s="92"/>
+      <c r="C30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="27" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="79" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="65"/>
-      <c r="C31" s="66" t="s">
+      <c r="B31" s="80"/>
+      <c r="C31" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="67"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="66" t="s">
+      <c r="D31" s="82"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="G31" s="67"/>
-      <c r="H31" s="68"/>
-    </row>
-    <row r="32" spans="1:8" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="83"/>
+    </row>
+    <row r="32" spans="1:8" s="1" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
     </row>
     <row r="33" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="50" t="s">
+      <c r="A33" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B33" s="51"/>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="51"/>
-      <c r="F33" s="51"/>
-      <c r="G33" s="51"/>
-      <c r="H33" s="40"/>
+      <c r="B33" s="70"/>
+      <c r="C33" s="70"/>
+      <c r="D33" s="70"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="70"/>
+      <c r="G33" s="70"/>
+      <c r="H33" s="48"/>
     </row>
     <row r="34" spans="1:8" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="52" t="s">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="D34" s="53"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="52" t="s">
+      <c r="D34" s="75"/>
+      <c r="E34" s="68"/>
+      <c r="F34" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="G34" s="53"/>
-      <c r="H34" s="49"/>
+      <c r="G34" s="75"/>
+      <c r="H34" s="68"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="10" t="s">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="10" t="s">
+      <c r="F35" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G35" s="10" t="s">
+      <c r="G35" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="H35" s="14" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="45" t="s">
+      <c r="A36" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="54"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
+      <c r="B36" s="98"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="55"/>
-      <c r="B37" s="56"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
+      <c r="A37" s="99"/>
+      <c r="B37" s="100"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="57" t="s">
+      <c r="A38" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="58"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
+      <c r="B38" s="101"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
     </row>
     <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="45" t="s">
+      <c r="A39" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="46"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
+      <c r="B39" s="102"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="42" t="s">
+      <c r="A40" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="B40" s="44"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
+      <c r="B40" s="65"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="42" t="s">
+      <c r="A41" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B41" s="44"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="42" t="s">
+      <c r="A42" s="61" t="s">
         <v>31</v>
       </c>
-      <c r="B42" s="44"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="7"/>
+      <c r="B42" s="65"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="42" t="s">
+      <c r="A43" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="B43" s="44"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
+      <c r="B43" s="65"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="42" t="s">
+      <c r="A44" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="44"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6"/>
+      <c r="B44" s="65"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="42" t="s">
+      <c r="A45" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="B45" s="44"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
+      <c r="B45" s="65"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="B46" s="44"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
+      <c r="B46" s="65"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="42" t="s">
+      <c r="A47" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="B47" s="44"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
     </row>
     <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="42" t="s">
+      <c r="A48" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="B48" s="44"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
+      <c r="B48" s="65"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
     </row>
     <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="42" t="s">
+      <c r="A49" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="B49" s="44"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-    </row>
-    <row r="50" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="42" t="s">
+      <c r="B49" s="65"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B50" s="44"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="35"/>
-      <c r="F50" s="35"/>
-      <c r="G50" s="35"/>
-      <c r="H50" s="35"/>
-    </row>
-    <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="42" t="s">
+      <c r="B50" s="65"/>
+      <c r="C50" s="39"/>
+      <c r="D50" s="39"/>
+      <c r="E50" s="39"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="39"/>
+      <c r="H50" s="39"/>
+    </row>
+    <row r="51" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="43"/>
-      <c r="C51" s="32"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="33"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="34"/>
-    </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="42" t="s">
+      <c r="B51" s="62"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="37"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
+    </row>
+    <row r="52" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="B52" s="43"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="29"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="31"/>
-    </row>
-    <row r="53" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="42" t="s">
+      <c r="B52" s="62"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="34"/>
+      <c r="E52" s="34"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="35"/>
+    </row>
+    <row r="53" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="B53" s="44"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="27"/>
-      <c r="H53" s="28"/>
+      <c r="B53" s="65"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="32"/>
     </row>
     <row r="54" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="45" t="s">
+      <c r="A54" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="B54" s="46"/>
-      <c r="C54" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="16"/>
+      <c r="B54" s="102"/>
+      <c r="C54" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="20"/>
     </row>
     <row r="55" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="47" t="s">
+      <c r="A55" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="B55" s="48"/>
-      <c r="C55" s="48"/>
-      <c r="D55" s="48"/>
-      <c r="E55" s="48"/>
-      <c r="F55" s="48"/>
-      <c r="G55" s="48"/>
-      <c r="H55" s="49"/>
+      <c r="B55" s="67"/>
+      <c r="C55" s="67"/>
+      <c r="D55" s="67"/>
+      <c r="E55" s="67"/>
+      <c r="F55" s="67"/>
+      <c r="G55" s="67"/>
+      <c r="H55" s="68"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A56" s="44" t="s">
+      <c r="A56" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="B56" s="44"/>
-      <c r="C56" s="44"/>
-      <c r="D56" s="44"/>
-      <c r="E56" s="44" t="s">
+      <c r="B56" s="65"/>
+      <c r="C56" s="65"/>
+      <c r="D56" s="65"/>
+      <c r="E56" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="F56" s="44"/>
-      <c r="G56" s="44"/>
-      <c r="H56" s="44"/>
+      <c r="F56" s="65"/>
+      <c r="G56" s="65"/>
+      <c r="H56" s="65"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="B58" s="41"/>
-      <c r="C58" s="41"/>
-      <c r="D58" s="41"/>
-      <c r="E58" s="41" t="s">
+      <c r="B58" s="60"/>
+      <c r="C58" s="60"/>
+      <c r="D58" s="60"/>
+      <c r="E58" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="F58" s="41"/>
-      <c r="G58" s="41"/>
-      <c r="H58" s="41"/>
+      <c r="F58" s="60"/>
+      <c r="G58" s="60"/>
+      <c r="H58" s="60"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="E56:H56"/>
+    <mergeCell ref="E58:H58"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A36:B37"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A9:H9"/>
     <mergeCell ref="E2:H4"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="F31:H31"/>
@@ -2288,41 +4338,6 @@
     <mergeCell ref="C25:E25"/>
     <mergeCell ref="F25:H25"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A36:B37"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="E56:H56"/>
-    <mergeCell ref="E58:H58"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A43:B43"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.28999999999999998" right="0.15748031496062992" top="0.2" bottom="0.21" header="0.15748031496062992" footer="0"/>
@@ -2330,4 +4345,1478 @@
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4CA5C6-71CF-4CF6-A8A7-B72F7074127B}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:H61"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" style="8"/>
+    <col min="2" max="2" width="9" style="8" customWidth="1"/>
+    <col min="3" max="8" width="13.7109375" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E2" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+    </row>
+    <row r="3" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+    </row>
+    <row r="4" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E5" s="84" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="86" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="86"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="97"/>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97"/>
+    </row>
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="16"/>
+      <c r="E7" s="84" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
+    </row>
+    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="D8" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="45"/>
+      <c r="F8" s="85" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="85"/>
+      <c r="H8" s="85"/>
+    </row>
+    <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A9" s="49"/>
+      <c r="B9" s="16"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+    </row>
+    <row r="10" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="78" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="78"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="78"/>
+      <c r="H10" s="78"/>
+    </row>
+    <row r="11" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="68"/>
+    </row>
+    <row r="12" spans="1:8" ht="2.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="96" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="96"/>
+      <c r="C13" s="96"/>
+      <c r="D13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+    </row>
+    <row r="14" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="93"/>
+      <c r="B20" s="93"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="94" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="95"/>
+      <c r="C25" s="79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="80"/>
+      <c r="E25" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="29"/>
+      <c r="G25" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="21"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="75"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="75"/>
+      <c r="H26" s="68"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H27" s="28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="87"/>
+      <c r="C28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="88"/>
+      <c r="B29" s="89"/>
+      <c r="C29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="90"/>
+      <c r="C30" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="91"/>
+      <c r="B31" s="92"/>
+      <c r="C31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="79" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="80"/>
+      <c r="C32" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="82"/>
+      <c r="E32" s="83"/>
+      <c r="F32" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="82"/>
+      <c r="H32" s="83"/>
+    </row>
+    <row r="33" spans="1:8" s="1" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
+      <c r="D34" s="70"/>
+      <c r="E34" s="70"/>
+      <c r="F34" s="70"/>
+      <c r="G34" s="70"/>
+      <c r="H34" s="48"/>
+    </row>
+    <row r="35" spans="1:8" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="75"/>
+      <c r="E35" s="68"/>
+      <c r="F35" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" s="75"/>
+      <c r="H35" s="68"/>
+    </row>
+    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="98"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="99"/>
+      <c r="B38" s="100"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="79" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" s="101"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="26"/>
+    </row>
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="102"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+    </row>
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="65"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+    </row>
+    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="B42" s="65"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+    </row>
+    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="61" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="65"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+    </row>
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="61" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="65"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="65"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="103" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="65"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="61" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" s="65"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="103" t="s">
+        <v>56</v>
+      </c>
+      <c r="B48" s="104"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="B49" s="65"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="61" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" s="65"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+    </row>
+    <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" s="65"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+    </row>
+    <row r="52" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="61" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="65"/>
+      <c r="C52" s="39"/>
+      <c r="D52" s="39"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="39"/>
+    </row>
+    <row r="53" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="B53" s="62"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="37"/>
+      <c r="E53" s="37"/>
+      <c r="F53" s="36"/>
+      <c r="G53" s="37"/>
+      <c r="H53" s="38"/>
+    </row>
+    <row r="54" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54" s="62"/>
+      <c r="C54" s="33"/>
+      <c r="D54" s="34"/>
+      <c r="E54" s="34"/>
+      <c r="F54" s="33"/>
+      <c r="G54" s="34"/>
+      <c r="H54" s="35"/>
+    </row>
+    <row r="55" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="61" t="s">
+        <v>40</v>
+      </c>
+      <c r="B55" s="65"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="30"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="32"/>
+    </row>
+    <row r="56" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="71" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" s="102"/>
+      <c r="C56" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="20"/>
+    </row>
+    <row r="57" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="66" t="s">
+        <v>37</v>
+      </c>
+      <c r="B57" s="67"/>
+      <c r="C57" s="67"/>
+      <c r="D57" s="67"/>
+      <c r="E57" s="67"/>
+      <c r="F57" s="67"/>
+      <c r="G57" s="67"/>
+      <c r="H57" s="68"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" s="65"/>
+      <c r="C58" s="65"/>
+      <c r="D58" s="65"/>
+      <c r="E58" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="F58" s="65"/>
+      <c r="G58" s="65"/>
+      <c r="H58" s="65"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" s="60"/>
+      <c r="C60" s="60"/>
+      <c r="D60" s="60"/>
+      <c r="E60" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="F60" s="60"/>
+      <c r="G60" s="60"/>
+      <c r="H60" s="60"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="9"/>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="9"/>
+      <c r="H61" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="E2:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="A28:B29"/>
+    <mergeCell ref="A30:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="A37:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="E60:H60"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="E58:H58"/>
+    <mergeCell ref="A49:B49"/>
+  </mergeCells>
+  <pageMargins left="0.28999999999999998" right="0.15748031496062992" top="0.2" bottom="0.21" header="0.15748031496062992" footer="0"/>
+  <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B75180-5C0C-45CC-A1A3-0E6643670006}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:I60"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" style="8"/>
+    <col min="2" max="2" width="9" style="8" customWidth="1"/>
+    <col min="3" max="8" width="13.7109375" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E2" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+    </row>
+    <row r="3" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+    </row>
+    <row r="4" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E5" s="84" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+    </row>
+    <row r="6" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="86" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="86"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+    </row>
+    <row r="7" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="105" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="105"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="54"/>
+    </row>
+    <row r="8" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="105" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="105"/>
+    </row>
+    <row r="9" spans="1:9" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="106" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="106"/>
+      <c r="C9" s="52"/>
+      <c r="D9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="107" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="107"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+    </row>
+    <row r="11" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="68"/>
+    </row>
+    <row r="12" spans="1:9" ht="2.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="96" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="96"/>
+      <c r="C13" s="96"/>
+      <c r="D13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+    </row>
+    <row r="14" spans="1:9" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="93"/>
+      <c r="B20" s="93"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="94" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="95"/>
+      <c r="C25" s="79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="80"/>
+      <c r="E25" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="29"/>
+      <c r="G25" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="21"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="75"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="75"/>
+      <c r="H26" s="68"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H27" s="28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="87"/>
+      <c r="C28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="88"/>
+      <c r="B29" s="89"/>
+      <c r="C29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="90"/>
+      <c r="C30" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="91"/>
+      <c r="B31" s="92"/>
+      <c r="C31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="79" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="80"/>
+      <c r="C32" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="82"/>
+      <c r="E32" s="83"/>
+      <c r="F32" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="82"/>
+      <c r="H32" s="83"/>
+    </row>
+    <row r="33" spans="1:8" s="1" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
+      <c r="D34" s="70"/>
+      <c r="E34" s="70"/>
+      <c r="F34" s="70"/>
+      <c r="G34" s="70"/>
+      <c r="H34" s="48"/>
+    </row>
+    <row r="35" spans="1:8" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="75"/>
+      <c r="E35" s="68"/>
+      <c r="F35" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" s="75"/>
+      <c r="H35" s="68"/>
+    </row>
+    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="98"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="99"/>
+      <c r="B38" s="100"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="79" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" s="101"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="26"/>
+    </row>
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="102"/>
+      <c r="C40" s="56">
+        <v>1</v>
+      </c>
+      <c r="D40" s="56">
+        <v>1</v>
+      </c>
+      <c r="E40" s="56"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+    </row>
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="65"/>
+      <c r="C41" s="57">
+        <v>1</v>
+      </c>
+      <c r="D41" s="57">
+        <v>1</v>
+      </c>
+      <c r="E41" s="57">
+        <v>1</v>
+      </c>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+    </row>
+    <row r="42" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="103" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="104"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+    </row>
+    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="61" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="65"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+    </row>
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="61" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="65"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="65"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="61" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" s="65"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="B47" s="65"/>
+      <c r="C47" s="56">
+        <v>2</v>
+      </c>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48" s="65"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="61" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" s="65"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B50" s="65"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+    </row>
+    <row r="51" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="61" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" s="65"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="39"/>
+    </row>
+    <row r="52" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="B52" s="62"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="37"/>
+      <c r="E52" s="37"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="37"/>
+      <c r="H52" s="38"/>
+    </row>
+    <row r="53" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="B53" s="62"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="34"/>
+      <c r="E53" s="34"/>
+      <c r="F53" s="33"/>
+      <c r="G53" s="34"/>
+      <c r="H53" s="35"/>
+    </row>
+    <row r="54" spans="1:8" s="6" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="61" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="65"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="30"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="32"/>
+    </row>
+    <row r="55" spans="1:8" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="71" t="s">
+        <v>35</v>
+      </c>
+      <c r="B55" s="102"/>
+      <c r="C55" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="20"/>
+    </row>
+    <row r="56" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="66" t="s">
+        <v>37</v>
+      </c>
+      <c r="B56" s="67"/>
+      <c r="C56" s="67"/>
+      <c r="D56" s="67"/>
+      <c r="E56" s="67"/>
+      <c r="F56" s="67"/>
+      <c r="G56" s="67"/>
+      <c r="H56" s="68"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" s="65"/>
+      <c r="C57" s="65"/>
+      <c r="D57" s="65"/>
+      <c r="E57" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="F57" s="65"/>
+      <c r="G57" s="65"/>
+      <c r="H57" s="65"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="60"/>
+      <c r="C59" s="60"/>
+      <c r="D59" s="60"/>
+      <c r="E59" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="F59" s="60"/>
+      <c r="G59" s="60"/>
+      <c r="H59" s="60"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="9"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="E59:H59"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="E57:H57"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="A37:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="A28:B29"/>
+    <mergeCell ref="A30:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E2:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A8:B8"/>
+  </mergeCells>
+  <pageMargins left="0.28999999999999998" right="0.15748031496062992" top="0.2" bottom="0.21" header="0.15748031496062992" footer="0"/>
+  <pageSetup paperSize="9" scale="79" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>